<commit_message>
update code using numba and optimize time running
</commit_message>
<xml_diff>
--- a/result/C1_Test.xlsx
+++ b/result/C1_Test.xlsx
@@ -649,112 +649,112 @@
         <v>1</v>
       </c>
       <c r="B4" s="3">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C4" s="3">
-        <v>1529.43</v>
+        <v>4020.01</v>
       </c>
       <c r="D4" s="3">
-        <v>20272.4</v>
+        <v>35757.54</v>
       </c>
       <c r="E4" s="3">
-        <v>0.12</v>
+        <v>0.24</v>
       </c>
       <c r="F4" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3">
-        <v>1192.38</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3">
-        <v>10681.57</v>
+        <v>0</v>
       </c>
       <c r="I4" s="3">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3">
-        <v>1334.82</v>
+        <v>0</v>
       </c>
       <c r="L4" s="3">
-        <v>6753.28</v>
+        <v>0</v>
       </c>
       <c r="M4" s="3">
-        <v>0.21</v>
+        <v>0</v>
       </c>
       <c r="N4" s="3">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O4" s="3">
-        <v>1060.94</v>
+        <v>0</v>
       </c>
       <c r="P4" s="3">
-        <v>1894.02</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="R4" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="S4" s="3">
-        <v>1194.06</v>
+        <v>0</v>
       </c>
       <c r="T4" s="3">
-        <v>14579.21</v>
+        <v>0</v>
       </c>
       <c r="U4" s="3">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="V4" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W4" s="3">
-        <v>1137.05</v>
+        <v>0</v>
       </c>
       <c r="X4" s="3">
-        <v>13736.86</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="3">
-        <v>1250.38</v>
+        <v>0</v>
       </c>
       <c r="AB4" s="3">
-        <v>14724.65</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="3">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="AD4" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AE4" s="3">
-        <v>1301.77</v>
+        <v>0</v>
       </c>
       <c r="AF4" s="3">
-        <v>11765.3</v>
+        <v>0</v>
       </c>
       <c r="AG4" s="3">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="AH4" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AI4" s="3">
-        <v>1163.46</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="3">
-        <v>7992.41</v>
+        <v>0</v>
       </c>
       <c r="AK4" s="3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -762,112 +762,112 @@
         <v>2</v>
       </c>
       <c r="B5" s="3">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C5" s="3">
-        <v>1417.39</v>
+        <v>3906</v>
       </c>
       <c r="D5" s="3">
-        <v>19229.2</v>
+        <v>34728.53</v>
       </c>
       <c r="E5" s="3">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="F5" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3">
-        <v>1288.04</v>
+        <v>0</v>
       </c>
       <c r="H5" s="3">
-        <v>8763.379999999999</v>
+        <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="J5" s="3">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K5" s="3">
-        <v>1117.35</v>
+        <v>0</v>
       </c>
       <c r="L5" s="3">
-        <v>3976.23</v>
+        <v>0</v>
       </c>
       <c r="M5" s="3">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="N5" s="3">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O5" s="3">
-        <v>1097.23</v>
+        <v>0</v>
       </c>
       <c r="P5" s="3">
-        <v>2064.16</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="R5" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="S5" s="3">
-        <v>1165.62</v>
+        <v>0</v>
       </c>
       <c r="T5" s="3">
-        <v>10710.73</v>
+        <v>0</v>
       </c>
       <c r="U5" s="3">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="V5" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W5" s="3">
-        <v>1197.35</v>
+        <v>0</v>
       </c>
       <c r="X5" s="3">
-        <v>14322.64</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="3">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="3">
-        <v>1159.57</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="3">
-        <v>10025.52</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="3">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="3">
-        <v>1132.47</v>
+        <v>0</v>
       </c>
       <c r="AF5" s="3">
-        <v>7916.95</v>
+        <v>0</v>
       </c>
       <c r="AG5" s="3">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="AH5" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AI5" s="3">
-        <v>1068.14</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="3">
-        <v>4476.01</v>
+        <v>0</v>
       </c>
       <c r="AK5" s="3">
-        <v>0.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:37">
@@ -875,112 +875,112 @@
         <v>3</v>
       </c>
       <c r="B6" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3">
-        <v>1207.53</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3">
-        <v>16835.83</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3">
-        <v>1203.77</v>
+        <v>0</v>
       </c>
       <c r="H6" s="3">
-        <v>12003.57</v>
+        <v>0</v>
       </c>
       <c r="I6" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3">
-        <v>1156.99</v>
+        <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>4342.89</v>
+        <v>0</v>
       </c>
       <c r="M6" s="3">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="N6" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O6" s="3">
-        <v>1113.01</v>
+        <v>0</v>
       </c>
       <c r="P6" s="3">
-        <v>2127.16</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="R6" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="S6" s="3">
-        <v>1199.13</v>
+        <v>0</v>
       </c>
       <c r="T6" s="3">
-        <v>16516.7</v>
+        <v>0</v>
       </c>
       <c r="U6" s="3">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="V6" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W6" s="3">
-        <v>1170.56</v>
+        <v>0</v>
       </c>
       <c r="X6" s="3">
-        <v>11161.34</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="3">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="3">
-        <v>1204.34</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="3">
-        <v>14220.38</v>
+        <v>0</v>
       </c>
       <c r="AC6" s="3">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="AD6" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="3">
-        <v>1146.93</v>
+        <v>0</v>
       </c>
       <c r="AF6" s="3">
-        <v>10444.86</v>
+        <v>0</v>
       </c>
       <c r="AG6" s="3">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="AH6" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AI6" s="3">
-        <v>1242.44</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="3">
-        <v>8176.89</v>
+        <v>0</v>
       </c>
       <c r="AK6" s="3">
-        <v>0.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -988,112 +988,112 @@
         <v>4</v>
       </c>
       <c r="B7" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C7" s="3">
-        <v>1066.12</v>
+        <v>0</v>
       </c>
       <c r="D7" s="3">
-        <v>14072.93</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3">
-        <v>1301.69</v>
+        <v>0</v>
       </c>
       <c r="H7" s="3">
-        <v>11138.28</v>
+        <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J7" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K7" s="3">
-        <v>1187.55</v>
+        <v>0</v>
       </c>
       <c r="L7" s="3">
-        <v>4961.11</v>
+        <v>0</v>
       </c>
       <c r="M7" s="3">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="N7" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O7" s="3">
-        <v>1145.99</v>
+        <v>0</v>
       </c>
       <c r="P7" s="3">
-        <v>2789.39</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="3">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="R7" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="S7" s="3">
-        <v>1275.59</v>
+        <v>0</v>
       </c>
       <c r="T7" s="3">
-        <v>13088.51</v>
+        <v>0</v>
       </c>
       <c r="U7" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="V7" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W7" s="3">
-        <v>1243.31</v>
+        <v>0</v>
       </c>
       <c r="X7" s="3">
-        <v>13171.81</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="3">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="3">
-        <v>1128.2</v>
+        <v>0</v>
       </c>
       <c r="AB7" s="3">
-        <v>11644.95</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="3">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="AD7" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AE7" s="3">
-        <v>1072.25</v>
+        <v>0</v>
       </c>
       <c r="AF7" s="3">
-        <v>7312.34</v>
+        <v>0</v>
       </c>
       <c r="AG7" s="3">
-        <v>0.32</v>
+        <v>0</v>
       </c>
       <c r="AH7" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AI7" s="3">
-        <v>1117.9</v>
+        <v>0</v>
       </c>
       <c r="AJ7" s="3">
-        <v>7704.16</v>
+        <v>0</v>
       </c>
       <c r="AK7" s="3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -1101,112 +1101,112 @@
         <v>5</v>
       </c>
       <c r="B8" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C8" s="3">
-        <v>1218.51</v>
+        <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>13223.52</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3">
-        <v>1268.54</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3">
-        <v>11313.69</v>
+        <v>0</v>
       </c>
       <c r="I8" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3">
-        <v>1172.27</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3">
-        <v>6488.89</v>
+        <v>0</v>
       </c>
       <c r="M8" s="3">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O8" s="3">
-        <v>1133.64</v>
+        <v>0</v>
       </c>
       <c r="P8" s="3">
-        <v>1756.79</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="R8" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>1249.58</v>
+        <v>0</v>
       </c>
       <c r="T8" s="3">
-        <v>16345.32</v>
+        <v>0</v>
       </c>
       <c r="U8" s="3">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="W8" s="3">
-        <v>1166.96</v>
+        <v>0</v>
       </c>
       <c r="X8" s="3">
-        <v>13221.7</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="3">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="3">
-        <v>1265.41</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="3">
-        <v>11801.53</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="3">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="3">
-        <v>1233.97</v>
+        <v>0</v>
       </c>
       <c r="AF8" s="3">
-        <v>13173.47</v>
+        <v>0</v>
       </c>
       <c r="AG8" s="3">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="AH8" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AI8" s="3">
-        <v>1227.33</v>
+        <v>0</v>
       </c>
       <c r="AJ8" s="3">
-        <v>8791.84</v>
+        <v>0</v>
       </c>
       <c r="AK8" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:37">
@@ -1214,112 +1214,112 @@
         <v>6</v>
       </c>
       <c r="B9" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="C9" s="3">
-        <v>1262.45</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3">
-        <v>19158.57</v>
+        <v>0</v>
       </c>
       <c r="E9" s="3">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G9" s="3">
-        <v>1202.63</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3">
-        <v>7799.82</v>
+        <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="J9" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K9" s="3">
-        <v>1280.1</v>
+        <v>0</v>
       </c>
       <c r="L9" s="3">
-        <v>6146.22</v>
+        <v>0</v>
       </c>
       <c r="M9" s="3">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="N9" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O9" s="3">
-        <v>1239.73</v>
+        <v>0</v>
       </c>
       <c r="P9" s="3">
-        <v>3023.95</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="3">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="R9" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S9" s="3">
-        <v>1220.5</v>
+        <v>0</v>
       </c>
       <c r="T9" s="3">
-        <v>14627.79</v>
+        <v>0</v>
       </c>
       <c r="U9" s="3">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="V9" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W9" s="3">
-        <v>1230.09</v>
+        <v>0</v>
       </c>
       <c r="X9" s="3">
-        <v>15133.5</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="3">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AA9" s="3">
-        <v>1348.99</v>
+        <v>0</v>
       </c>
       <c r="AB9" s="3">
-        <v>14288.9</v>
+        <v>0</v>
       </c>
       <c r="AC9" s="3">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="3">
-        <v>1161.91</v>
+        <v>0</v>
       </c>
       <c r="AF9" s="3">
-        <v>7830.4</v>
+        <v>0</v>
       </c>
       <c r="AG9" s="3">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="AH9" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AI9" s="3">
-        <v>1280.01</v>
+        <v>0</v>
       </c>
       <c r="AJ9" s="3">
-        <v>9603.43</v>
+        <v>0</v>
       </c>
       <c r="AK9" s="3">
-        <v>0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -1327,112 +1327,112 @@
         <v>7</v>
       </c>
       <c r="B10" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C10" s="3">
-        <v>1224.37</v>
+        <v>0</v>
       </c>
       <c r="D10" s="3">
-        <v>16229.9</v>
+        <v>0</v>
       </c>
       <c r="E10" s="3">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="F10" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3">
-        <v>1369.57</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3">
-        <v>12422.24</v>
+        <v>0</v>
       </c>
       <c r="I10" s="3">
-        <v>0.21</v>
+        <v>0</v>
       </c>
       <c r="J10" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3">
-        <v>1217.68</v>
+        <v>0</v>
       </c>
       <c r="L10" s="3">
-        <v>5977.15</v>
+        <v>0</v>
       </c>
       <c r="M10" s="3">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="N10" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O10" s="3">
-        <v>1210.98</v>
+        <v>0</v>
       </c>
       <c r="P10" s="3">
-        <v>3750.83</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="R10" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="S10" s="3">
-        <v>1258.29</v>
+        <v>0</v>
       </c>
       <c r="T10" s="3">
-        <v>14389.38</v>
+        <v>0</v>
       </c>
       <c r="U10" s="3">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="V10" s="3">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="W10" s="3">
-        <v>1349.67</v>
+        <v>0</v>
       </c>
       <c r="X10" s="3">
-        <v>14532.33</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="3">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="3">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="3">
-        <v>1296.09</v>
+        <v>0</v>
       </c>
       <c r="AB10" s="3">
-        <v>14788.03</v>
+        <v>0</v>
       </c>
       <c r="AC10" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="AD10" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AE10" s="3">
-        <v>1197.62</v>
+        <v>0</v>
       </c>
       <c r="AF10" s="3">
-        <v>10925.03</v>
+        <v>0</v>
       </c>
       <c r="AG10" s="3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AH10" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AI10" s="3">
-        <v>1119.18</v>
+        <v>0</v>
       </c>
       <c r="AJ10" s="3">
-        <v>7405.53</v>
+        <v>0</v>
       </c>
       <c r="AK10" s="3">
-        <v>0.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -1440,112 +1440,112 @@
         <v>8</v>
       </c>
       <c r="B11" s="3">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3">
-        <v>1343.79</v>
+        <v>0</v>
       </c>
       <c r="D11" s="3">
-        <v>20654.04</v>
+        <v>0</v>
       </c>
       <c r="E11" s="3">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="F11" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3">
-        <v>1274.5</v>
+        <v>0</v>
       </c>
       <c r="H11" s="3">
-        <v>12789.5</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="J11" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K11" s="3">
-        <v>1136.57</v>
+        <v>0</v>
       </c>
       <c r="L11" s="3">
-        <v>5321.3</v>
+        <v>0</v>
       </c>
       <c r="M11" s="3">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="N11" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="O11" s="3">
-        <v>1154.79</v>
+        <v>0</v>
       </c>
       <c r="P11" s="3">
-        <v>2525.41</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="3">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="R11" s="3">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="S11" s="3">
-        <v>1497.07</v>
+        <v>0</v>
       </c>
       <c r="T11" s="3">
-        <v>22581.18</v>
+        <v>0</v>
       </c>
       <c r="U11" s="3">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="V11" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="W11" s="3">
-        <v>1330.44</v>
+        <v>0</v>
       </c>
       <c r="X11" s="3">
-        <v>16324.12</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="3">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="3">
-        <v>1210.53</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="3">
-        <v>14118.08</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="3">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="AD11" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AE11" s="3">
-        <v>1197.7</v>
+        <v>0</v>
       </c>
       <c r="AF11" s="3">
-        <v>12918.58</v>
+        <v>0</v>
       </c>
       <c r="AG11" s="3">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="AH11" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AI11" s="3">
-        <v>1121.19</v>
+        <v>0</v>
       </c>
       <c r="AJ11" s="3">
-        <v>5200.25</v>
+        <v>0</v>
       </c>
       <c r="AK11" s="3">
-        <v>0.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:37">
@@ -1553,112 +1553,112 @@
         <v>9</v>
       </c>
       <c r="B12" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="C12" s="3">
-        <v>1314.76</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3">
-        <v>20108.17</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="F12" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3">
-        <v>1243.55</v>
+        <v>0</v>
       </c>
       <c r="H12" s="3">
-        <v>11462.2</v>
+        <v>0</v>
       </c>
       <c r="I12" s="3">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K12" s="3">
-        <v>1266.55</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3">
-        <v>6753.39</v>
+        <v>0</v>
       </c>
       <c r="M12" s="3">
-        <v>0.33</v>
+        <v>0</v>
       </c>
       <c r="N12" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O12" s="3">
-        <v>1291.39</v>
+        <v>0</v>
       </c>
       <c r="P12" s="3">
-        <v>3370.05</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="3">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="R12" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S12" s="3">
-        <v>1326.29</v>
+        <v>0</v>
       </c>
       <c r="T12" s="3">
-        <v>20522.32</v>
+        <v>0</v>
       </c>
       <c r="U12" s="3">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="V12" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="W12" s="3">
-        <v>1204.92</v>
+        <v>0</v>
       </c>
       <c r="X12" s="3">
-        <v>14050.1</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="3">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="3">
-        <v>1156.35</v>
+        <v>0</v>
       </c>
       <c r="AB12" s="3">
-        <v>12074.71</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="3">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="3">
-        <v>1138.4</v>
+        <v>0</v>
       </c>
       <c r="AF12" s="3">
-        <v>11719.67</v>
+        <v>0</v>
       </c>
       <c r="AG12" s="3">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="AH12" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AI12" s="3">
-        <v>1059.53</v>
+        <v>0</v>
       </c>
       <c r="AJ12" s="3">
-        <v>5796.79</v>
+        <v>0</v>
       </c>
       <c r="AK12" s="3">
-        <v>0.14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:37">
@@ -1666,112 +1666,112 @@
         <v>10</v>
       </c>
       <c r="B13" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C13" s="3">
-        <v>1203.09</v>
+        <v>0</v>
       </c>
       <c r="D13" s="3">
-        <v>15948.02</v>
+        <v>0</v>
       </c>
       <c r="E13" s="3">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="F13" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G13" s="3">
-        <v>1219.44</v>
+        <v>0</v>
       </c>
       <c r="H13" s="3">
-        <v>11102.83</v>
+        <v>0</v>
       </c>
       <c r="I13" s="3">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J13" s="3">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K13" s="3">
-        <v>1180.98</v>
+        <v>0</v>
       </c>
       <c r="L13" s="3">
-        <v>4554.8</v>
+        <v>0</v>
       </c>
       <c r="M13" s="3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="N13" s="3">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O13" s="3">
-        <v>1171.92</v>
+        <v>0</v>
       </c>
       <c r="P13" s="3">
-        <v>2799.37</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="R13" s="3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="S13" s="3">
-        <v>1308.55</v>
+        <v>0</v>
       </c>
       <c r="T13" s="3">
-        <v>16528.7</v>
+        <v>0</v>
       </c>
       <c r="U13" s="3">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="V13" s="3">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="W13" s="3">
-        <v>1207.25</v>
+        <v>0</v>
       </c>
       <c r="X13" s="3">
-        <v>15038.54</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="3">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="3">
-        <v>1115.11</v>
+        <v>0</v>
       </c>
       <c r="AB13" s="3">
-        <v>11522.83</v>
+        <v>0</v>
       </c>
       <c r="AC13" s="3">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="AD13" s="3">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="3">
-        <v>1128.8</v>
+        <v>0</v>
       </c>
       <c r="AF13" s="3">
-        <v>11075.29</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AH13" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AI13" s="3">
-        <v>1183.14</v>
+        <v>0</v>
       </c>
       <c r="AJ13" s="3">
-        <v>6965.42</v>
+        <v>0</v>
       </c>
       <c r="AK13" s="3">
-        <v>0.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:37">
@@ -1779,112 +1779,112 @@
         <v>15</v>
       </c>
       <c r="B14" s="3">
-        <v>15.8</v>
+        <v>4.8</v>
       </c>
       <c r="C14" s="3">
-        <v>1278.744</v>
+        <v>792.601</v>
       </c>
       <c r="D14" s="3">
-        <v>17573.258</v>
+        <v>7048.607000000001</v>
       </c>
       <c r="E14" s="3">
-        <v>0.121</v>
+        <v>0.034</v>
       </c>
       <c r="F14" s="3">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3">
-        <v>1256.411</v>
+        <v>0</v>
       </c>
       <c r="H14" s="3">
-        <v>10947.708</v>
+        <v>0</v>
       </c>
       <c r="I14" s="3">
-        <v>0.163</v>
+        <v>0</v>
       </c>
       <c r="J14" s="3">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K14" s="3">
-        <v>1205.086</v>
+        <v>0</v>
       </c>
       <c r="L14" s="3">
-        <v>5527.526000000001</v>
+        <v>0</v>
       </c>
       <c r="M14" s="3">
-        <v>0.185</v>
+        <v>0</v>
       </c>
       <c r="N14" s="3">
-        <v>12.1</v>
+        <v>0</v>
       </c>
       <c r="O14" s="3">
-        <v>1161.962</v>
+        <v>0</v>
       </c>
       <c r="P14" s="3">
-        <v>2610.113</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="3">
-        <v>0.118</v>
+        <v>0</v>
       </c>
       <c r="R14" s="3">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="S14" s="3">
-        <v>1269.468</v>
+        <v>0</v>
       </c>
       <c r="T14" s="3">
-        <v>15988.984</v>
+        <v>0</v>
       </c>
       <c r="U14" s="3">
-        <v>0.136</v>
+        <v>0</v>
       </c>
       <c r="V14" s="3">
-        <v>15.1</v>
+        <v>0</v>
       </c>
       <c r="W14" s="3">
-        <v>1223.76</v>
+        <v>0</v>
       </c>
       <c r="X14" s="3">
-        <v>14069.294</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="3">
-        <v>0.206</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="3">
-        <v>14.7</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="3">
-        <v>1213.497</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="3">
-        <v>12920.958</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="3">
-        <v>0.151</v>
+        <v>0</v>
       </c>
       <c r="AD14" s="3">
-        <v>14.1</v>
+        <v>0</v>
       </c>
       <c r="AE14" s="3">
-        <v>1171.182</v>
+        <v>0</v>
       </c>
       <c r="AF14" s="3">
-        <v>10508.189</v>
+        <v>0</v>
       </c>
       <c r="AG14" s="3">
-        <v>0.202</v>
+        <v>0</v>
       </c>
       <c r="AH14" s="3">
-        <v>13.3</v>
+        <v>0</v>
       </c>
       <c r="AI14" s="3">
-        <v>1158.232</v>
+        <v>0</v>
       </c>
       <c r="AJ14" s="3">
-        <v>7211.272999999999</v>
+        <v>0</v>
       </c>
       <c r="AK14" s="3">
-        <v>0.133</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>